<commit_message>
corrected mixers, splitter and rWGS
</commit_message>
<xml_diff>
--- a/case_studies/backbone/technologies.xlsx
+++ b/case_studies/backbone/technologies.xlsx
@@ -1,25 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD2C54C-403D-4BD3-9890-AEA9B5C13438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A6431C-3712-4B36-A5BF-1B5DFB9BEE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="1" r:id="rId1"/>
     <sheet name="new" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -527,7 +538,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -557,10 +568,10 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>946.41</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>946.41</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -607,7 +618,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>45.67</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -684,7 +695,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>39.950000000000003</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -711,16 +722,16 @@
         <v>0</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>515.12</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>515.12</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>38.840000000000003</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -755,13 +766,13 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>217</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -865,10 +876,10 @@
         <v>0</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>566</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>566</v>
       </c>
       <c r="O6">
         <v>0</v>
@@ -951,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -1019,10 +1030,10 @@
         <v>0</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>329</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>329</v>
       </c>
       <c r="O8">
         <v>0</v>

</xml_diff>

<commit_message>
modified carriers according to unit of measures
</commit_message>
<xml_diff>
--- a/case_studies/backbone/technologies.xlsx
+++ b/case_studies/backbone/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A6431C-3712-4B36-A5BF-1B5DFB9BEE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7D2231-425C-4586-A120-04EC10B4000F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28935" yWindow="-375" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="1" r:id="rId1"/>
@@ -710,7 +710,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>18.3</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>55.6</v>
       </c>
       <c r="J7">
         <v>0</v>

</xml_diff>